<commit_message>
SMTP Check and Update
</commit_message>
<xml_diff>
--- a/database/intern.xlsx
+++ b/database/intern.xlsx
@@ -17,16 +17,13 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -37,7 +34,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -45,21 +42,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -425,86 +413,86 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P4"/>
+  <dimension ref="A1:P5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>Login Email</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>Full Name</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>Staff ID</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>Role</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>Department</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>Designation</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>Joining Date</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>Phone</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>Personal Email</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>Base Salary/Fee</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>Paid/HRA</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>Workshop Status</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>Payment Status</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>Pan Number</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>Bank Account</t>
         </is>
@@ -564,12 +552,12 @@
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>Inactive</t>
+          <t>Active</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>Completed</t>
+          <t>Ongoing</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
@@ -635,19 +623,19 @@
         </is>
       </c>
       <c r="J3" t="n">
-        <v>0</v>
+        <v>30000</v>
       </c>
       <c r="K3" t="n">
         <v>0</v>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>Inactive</t>
+          <t>Active</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>Completed</t>
+          <t>Ongoing</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
@@ -713,19 +701,19 @@
         </is>
       </c>
       <c r="J4" t="n">
-        <v>0</v>
+        <v>30000</v>
       </c>
       <c r="K4" t="n">
         <v>0</v>
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>Inactive</t>
+          <t>Active</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>Completed</t>
+          <t>Ongoing</t>
         </is>
       </c>
       <c r="N4" t="inlineStr">
@@ -739,6 +727,84 @@
         </is>
       </c>
       <c r="P4" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>itn-it-sambriddhi@ems.com</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Sambriddhi Gotame</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>ITN-IT-002</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Intern</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>IT</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Cyber Security Intern</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>2026-05-04</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>+977 9762874330</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>samridhigotame13@gmail.com</t>
+        </is>
+      </c>
+      <c r="J5" t="n">
+        <v>0</v>
+      </c>
+      <c r="K5" t="n">
+        <v>0</v>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="O5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="P5" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>

</xml_diff>